<commit_message>
update the form changes
</commit_message>
<xml_diff>
--- a/JobsNVisa.xlsx
+++ b/JobsNVisa.xlsx
@@ -1,19 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29711"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_5C9FE1BAB08E69A0B11CDEB6F3FB1025970095F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2D9E994-7C4E-42C6-BD0C-283C90AE4E30}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Job_Seekers" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Post_Jobs" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Contacts" state="visible" r:id="rId6"/>
+    <sheet name="Job_Seekers" sheetId="1" r:id="rId1"/>
+    <sheet name="Post_Jobs" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>Full Name</t>
   </si>
@@ -39,6 +58,9 @@
     <t>Experience Years</t>
   </si>
   <si>
+    <t>Resume</t>
+  </si>
+  <si>
     <t>Message</t>
   </si>
   <si>
@@ -64,25 +86,19 @@
   </si>
   <si>
     <t>Sponsorship</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Subject</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -445,20 +461,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="6" width="15" customWidth="1"/>
-    <col min="7" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="40" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="7" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -488,18 +504,21 @@
       </c>
       <c r="J1" t="s">
         <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
@@ -509,78 +528,40 @@
     <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>